<commit_message>
Nawigacja, sortowanie uczestników i generowanie obsluga-egzaminu-rec
- index.html: przycisk Zaloguj się (link do /zaloguj-sie) w navbarze
- Admin login przeniesiony z /login na /panel-42
- Przyciski Wyloguj i Wróć na stronę główną – styl z pomarańczową obwódką
- Sortowanie uczestników kursu rosnąco wg daty zapisu (pierwszy = Lp. 1)
- Generowanie obsluga-egzaminu-rec: wypełnia arkusz DANE danymi kursu i uczestników
- Arkusze xlsx ustawiane na układ poziomy przy generowaniu
- Usunięto nieistniejący plik zestawienie-rec z listy dokumentów recert

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/documents/templates/obecnosc.xlsx
+++ b/backend/documents/templates/obecnosc.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pkarp\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projekty Programowanie\McMed\backend\documents\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{E74ACEBC-12E6-46D6-B100-711994732CEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FB624955-A625-4CE8-AE5D-4DED2E82711A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{FB624955-A625-4CE8-AE5D-4DED2E82711A}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -409,7 +409,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -747,16 +747,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{258629F4-1709-4C14-B0F8-AC569B41BB39}">
   <dimension ref="A1:N11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.140625" customWidth="1"/>
-    <col min="2" max="2" width="22.140625" customWidth="1"/>
-    <col min="3" max="13" width="5.5703125" customWidth="1"/>
-    <col min="14" max="14" width="34.7109375" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="14.1796875" customWidth="1"/>
+    <col min="2" max="2" width="22.1796875" customWidth="1"/>
+    <col min="3" max="13" width="5.54296875" customWidth="1"/>
+    <col min="14" max="14" width="34.7265625" customWidth="1"/>
+    <col min="15" max="15" width="9.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="13" t="s">
         <v>45</v>
@@ -772,7 +772,7 @@
       <c r="K1" s="13"/>
       <c r="L1" s="13"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -785,14 +785,14 @@
       <c r="K2" s="13"/>
       <c r="L2" s="13"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="B3" s="14" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="14"/>
       <c r="D3" s="14"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
@@ -836,7 +836,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
         <v>15</v>
       </c>
@@ -878,7 +878,7 @@
       </c>
       <c r="N5" s="9"/>
     </row>
-    <row r="6" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
         <v>27</v>
       </c>
@@ -920,7 +920,7 @@
       </c>
       <c r="N6" s="9"/>
     </row>
-    <row r="7" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
         <v>28</v>
       </c>
@@ -962,7 +962,7 @@
       </c>
       <c r="N7" s="9"/>
     </row>
-    <row r="8" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
         <v>29</v>
       </c>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="N8" s="9"/>
     </row>
-    <row r="9" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
         <v>30</v>
       </c>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="N9" s="9"/>
     </row>
-    <row r="10" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
         <v>31</v>
       </c>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="N10" s="9"/>
     </row>
-    <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>43</v>
       </c>

</xml_diff>